<commit_message>
docs: record saved procurement application and company signing step
</commit_message>
<xml_diff>
--- a/procurement/output/나라장터-신청준비.xlsx
+++ b/procurement/output/나라장터-신청준비.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>회사 미등록. 대표자 본인·사업자용 범용 공동인증서로 회사 신규 등록부터 진행</t>
+          <t>회사 미등록. 등기임원 계정으로 로그인 완료. 회사 명의 범용 공동인증서를 보유하며 회사 신규 등록부터 진행</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>입력안·증빙 목록·실적·원가·자금·평가 양식 준비. 실제 신청·투찰 미실행</t>
+          <t>입력안·증빙 목록·실적·원가·자금·평가 양식 준비. 실제 신청서 저장·재조회 완료, 전자서명 대기. 투찰 미실행</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>업종 후보</t>
+          <t>업종</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -811,12 +811,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>현재 관광사업등록증 DOC-07 직접 확인</t>
+          <t>현재 관광사업등록증 DOC-07과 실제 업종 검색 결과 일치</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>실제 신청 화면의 업종 코드 대조</t>
+          <t>신청서 저장·재조회 완료, 전자서명 대기</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>대표자 본인</t>
+          <t>등기임원 개인회원 계정</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>개인회원 미가입: 대표자 본인 회원가입·인증부터 필요</t>
+          <t>가입·로그인 완료: 실제 로그인과 사용자 답변 확인 / 실제 대표자는 별도 입력</t>
         </is>
       </c>
     </row>
@@ -979,12 +979,12 @@
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>실제 신청 뒤 기록</t>
+          <t>실제 송신 완료 뒤 기록</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>아직 신청하지 않음</t>
+          <t>임시저장 완료, 회사 공동인증서 전자서명 대기</t>
         </is>
       </c>
     </row>
@@ -1191,19 +1191,19 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>대리인 경로만</t>
+          <t>신청 역할별 요구</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>요구 확인 중</t>
         </is>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>사용자 확인: 대표자 본인 직접 신청</t>
+          <t>등기임원 계정. 신청자와 실제 대표자를 구분하고 화면의 실제 요구를 확인</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: diagnose unsupported bank certificate in procurement signing
</commit_message>
<xml_diff>
--- a/procurement/output/나라장터-신청준비.xlsx
+++ b/procurement/output/나라장터-신청준비.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>회사 미등록. 등기임원 계정으로 로그인 완료. 회사 명의 범용 공동인증서를 보유하며 회사 신규 등록부터 진행</t>
+          <t>회사 미등록. 등기임원 계정으로 로그인 완료. 표준 로컬 인증서는 은행보험용이어서 적합 인증수단 확인 대기</t>
         </is>
       </c>
     </row>
@@ -934,17 +934,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>회사 명의 사업자용 범용 공동인증서 보유(사용자 확인)</t>
+          <t>범용 보유라는 사용자 답변과 달리 표준 로컬 폴더의 실제 인증서는 사업자 은행보험용으로 확인. 별도 범용 또는 사업자용 금융인증서 보유 여부 확인 대기</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>사용자 보유 확인</t>
+          <t>공개 인증서와 나라장터 공식 허용 목록 대조</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>인증서 파일·비밀번호 미수집, 유효기간 확인 필요</t>
+          <t>표준 로컬 인증서 기간 유효, 용도 미허용. 비밀키 내용·비밀번호 미수집</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: prepare business financial certificate issuance decision
</commit_message>
<xml_diff>
--- a/procurement/output/나라장터-신청준비.xlsx
+++ b/procurement/output/나라장터-신청준비.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>회사 미등록. 등기임원 계정으로 로그인 완료. 표준 로컬 인증서는 은행보험용이어서 적합 인증수단 확인 대기</t>
+          <t>회사 미등록. 등기임원 계정으로 로그인 완료. 은행보험용 인증서만 보유해 기업금융인증서 1년 4,400원 신규 발급 비용 승인 대기</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>범용 보유라는 사용자 답변과 달리 표준 로컬 폴더의 실제 인증서는 사업자 은행보험용으로 확인. 별도 범용 또는 사업자용 금융인증서 보유 여부 확인 대기</t>
+          <t>현재 PC의 사업자 은행보험용 공동인증서만 보유(사용자 확인). 나라장터 서명에는 미허용. 사업자용 금융인증서 신규 발급 비용 승인 대기</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: record approved certificate fee and bank interaction checkpoint
</commit_message>
<xml_diff>
--- a/procurement/output/나라장터-신청준비.xlsx
+++ b/procurement/output/나라장터-신청준비.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>회사 미등록. 등기임원 계정으로 로그인 완료. 은행보험용 인증서만 보유해 기업금융인증서 1년 4,400원 신규 발급 비용 승인 대기</t>
+          <t>회사 미등록. 등기임원 계정으로 로그인 완료. 기업금융인증서 1년 4,400원 발급 승인 완료. 실제 발급·본인확인 대기</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>현재 PC의 사업자 은행보험용 공동인증서만 보유(사용자 확인). 나라장터 서명에는 미허용. 사업자용 금융인증서 신규 발급 비용 승인 대기</t>
+          <t>현재 PC의 은행보험용 공동인증서만 보유. KB국민은행 기업금융인증서 1년·4,400원 발급 승인 완료. 실제 발급과 사용자 본인확인 대기</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: record reported financial certificate issuance and login recovery
</commit_message>
<xml_diff>
--- a/procurement/output/나라장터-신청준비.xlsx
+++ b/procurement/output/나라장터-신청준비.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>회사 미등록. 등기임원 계정으로 로그인 완료. 기업금융인증서 1년 4,400원 발급 승인 완료. 실제 발급·본인확인 대기</t>
+          <t>2026-10-21 기업금융인증서 발급 완료를 사용자 확인. 회사 신청서는 저장 상태이며 새 브라우저에서 재로그인 대기</t>
         </is>
       </c>
     </row>
@@ -934,17 +934,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>현재 PC의 은행보험용 공동인증서만 보유. KB국민은행 기업금융인증서 1년·4,400원 발급 승인 완료. 실제 발급과 사용자 본인확인 대기</t>
+          <t>KB국민은행 기업금융인증서 발급 완료(2026-10-21 사용자 확인). 승인 범위는 1년·4,400원. 실제 인증서 선택·유효기간·전자서명은 미확인</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>공개 인증서와 나라장터 공식 허용 목록 대조</t>
+          <t>기업금융인증서 발급 완료를 사용자 확인</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>표준 로컬 인증서 기간 유효, 용도 미허용. 비밀키 내용·비밀번호 미수집</t>
+          <t>이전 은행용 공동인증서와 구분. 새 금융인증서 실제 선택·서명은 미확인. 비밀번호 미수집</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>가입·로그인 완료: 실제 로그인과 사용자 답변 확인 / 실제 대표자는 별도 입력</t>
+          <t>개인회원 가입 완료. 2026-10-21 새 Aside 세션에서 재로그인 대기 / 실제 대표자는 별도 입력</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record procurement submission and supporting document delivery
</commit_message>
<xml_diff>
--- a/procurement/output/나라장터-신청준비.xlsx
+++ b/procurement/output/나라장터-신청준비.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 기업금융인증서 발급 완료를 사용자 확인. 회사 신청서는 저장 상태이며 새 브라우저에서 재로그인 대기</t>
+          <t>2026-10-21 회사 금융인증서 서명·신청 송신·관광사업등록증 온라인 제출 완료. 서울지방조달청 심사 대기</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>입력안·증빙 목록·실적·원가·자금·평가 양식 준비. 실제 신청서 저장·재조회 완료, 전자서명 대기. 투찰 미실행</t>
+          <t>입력안·증빙 목록·실적·원가·자금·평가 양식 준비. 실제 신청 송신·증빙 제출 완료, 심사 대기. 투찰 미실행</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>신청서 저장·재조회 완료, 전자서명 대기</t>
+          <t>신청 송신·증빙 제출 완료, 심사 대기</t>
         </is>
       </c>
     </row>
@@ -934,17 +934,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>KB국민은행 기업금융인증서 발급 완료(2026-10-21 사용자 확인). 승인 범위는 1년·4,400원. 실제 인증서 선택·유효기간·전자서명은 미확인</t>
+          <t>KB국민은행 금융공공용 1년 기업금융인증서. YESKEY에서 회사명·사업자번호 일치와 유효기간 2027-10-21 확인. 사용자가 전자서명 완료</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>기업금융인증서 발급 완료를 사용자 확인</t>
+          <t>YESKEY 회사명·사업자번호·유효기간 확인 및 사용자 서명</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>이전 은행용 공동인증서와 구분. 새 금융인증서 실제 선택·서명은 미확인. 비밀번호 미수집</t>
+          <t>유효기간 2027-10-21. 비밀번호 미수집. 수수료 출금은 미확인</t>
         </is>
       </c>
     </row>
@@ -966,25 +966,29 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>개인회원 가입 완료. 2026-10-21 새 Aside 세션에서 재로그인 대기 / 실제 대표자는 별도 입력</t>
+          <t>등기임원 개인회원 가입·2026-10-21 재로그인 확인 / 실제 대표자는 별도 입력</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>접수번호</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n"/>
+          <t>신청 접수</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>실제 송신 완료 뒤 기록</t>
+          <t>서울지방조달청 접수 안내문</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>임시저장 완료, 회사 공동인증서 전자서명 대기</t>
+          <t>별도 접수번호는 미확인. 중복 신청 금지</t>
         </is>
       </c>
     </row>
@@ -994,15 +998,19 @@
           <t>승인 상태</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>대기</t>
+        </is>
+      </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>조달청 승인 화면</t>
+          <t>온라인 증빙 제출 후 실제 화면</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>등록증 확보 전 완료 표시 금지</t>
+          <t>등록 승인·등록증은 아직 미확인</t>
         </is>
       </c>
     </row>

</xml_diff>